<commit_message>
v1.5 gite bu isimle gönder
</commit_message>
<xml_diff>
--- a/3-Kutu_Tasarım_Kontrolu/0-Kural.xlsx
+++ b/3-Kutu_Tasarım_Kontrolu/0-Kural.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vande\Desktop\Tasarım_Kontrol\3-Kutu_Tasarım_Kontrolu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85848AAB-C6BC-4710-B919-9FB41548E454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5980DCC6-9A00-4670-BC0D-06CA37555118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1755" yWindow="9825" windowWidth="17175" windowHeight="12990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1320" yWindow="0" windowWidth="21795" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Referans_Alan_Adı</t>
   </si>
@@ -69,6 +69,24 @@
   </si>
   <si>
     <t>KKKIKIKIIKII (7843)</t>
+  </si>
+  <si>
+    <t>Ürün Adı</t>
+  </si>
+  <si>
+    <t>Adres</t>
+  </si>
+  <si>
+    <t>Dizayn No</t>
+  </si>
+  <si>
+    <t>Farmakod</t>
+  </si>
+  <si>
+    <t>ATC kodu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> G04BE03.</t>
   </si>
 </sst>
 </file>
@@ -423,7 +441,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
@@ -431,7 +449,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -439,7 +457,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -447,7 +465,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -455,10 +473,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>1505891</v>
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>